<commit_message>
Xadra xarajatlar: yuqori qavat o'quv xonasiga bambuk panel
Buyurtmachi chizmasidagi yuqori qavat o'quv xonasi (5.45 × 8.60 m):
bambuk panel 3 devorga 2.5 m balandlikda — doska devori, orqa devor va
eshikli uzun devor (eshik o'rni ayiriladi). Panel balandligi «Narxlar»
varag'ida alohida katak. Jami 28 571.58 $.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0121VSEFiRNp3h6KMycRzKQh
</commit_message>
<xml_diff>
--- a/xadra-filiali/hisob/Xadra_2-qavat_xarajatlar_v1.0.xlsx
+++ b/xadra-filiali/hisob/Xadra_2-qavat_xarajatlar_v1.0.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="188">
   <si>
     <t xml:space="preserve">PDP Academy · Xadra filiali — 2-qavat: xarajatlar, xonalar bo'yicha</t>
   </si>
@@ -90,7 +90,7 @@
     <t xml:space="preserve">7-xona</t>
   </si>
   <si>
-    <t xml:space="preserve">Yuqori qavat o'quv xonasi</t>
+    <t xml:space="preserve">Yuqori qavat o'quv xonasi (5.45 × 8.60)</t>
   </si>
   <si>
     <t xml:space="preserve">O'quv xonalari — jami</t>
@@ -243,6 +243,9 @@
     <t xml:space="preserve">Taxmin: poldan shiftgacha. Pastroq bo'lsa, shu katakka raqam yozing</t>
   </si>
   <si>
+    <t xml:space="preserve">Bambuk panel balandligi — yuqori qavat o'quv xonasi</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hisoblash qoidalari</t>
   </si>
   <si>
@@ -258,6 +261,9 @@
     <t xml:space="preserve">• Bambuk panel, poldan shiftgacha: o'quv xonalarida doska devori va orqa devor (interaktiv doska orqasi ayirilmagan); ofis xonalarida ikkala uzun yon devor; CEO xonasida ikkita ichki kar devor, eshik o'rni ayiriladi. Derazali tashqi va shisha devorlarga qilinmaydi.</t>
   </si>
   <si>
+    <t xml:space="preserve">• Yuqori qavat o'quv xonasi (5.45 × 8.60 m, buyurtmachi chizmasi): bambuk panel 3 devorga, 2.5 m balandlikda — doska devori, orqa devor va eshikli uzun devor (eshik o'rni ayiriladi); derazali uzun devorga qilinmaydi.</t>
+  </si>
+  <si>
     <t xml:space="preserve">• Interaktiv doska: 7 ta shu qavat sinflariga va 1 ta yuqori qavatdagi o'quv xonasiga — jami 8 ta.</t>
   </si>
   <si>
@@ -564,10 +570,19 @@
     <t xml:space="preserve">Jami: Zinapoya</t>
   </si>
   <si>
+    <t xml:space="preserve">Doska devori (eni)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orqa devor (eni)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uzun devor (eshikli)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Yuqori qavatdagi o'quv xonasi uchun</t>
   </si>
   <si>
-    <t xml:space="preserve">Jami: Yuqori qavat o'quv xonasi</t>
+    <t xml:space="preserve">Jami: Yuqori qavat o'quv xonasi (5.45 × 8.60)</t>
   </si>
   <si>
     <t xml:space="preserve">JAMI (barcha xonalar)</t>
@@ -1216,43 +1231,43 @@
         <v>15</v>
       </c>
       <c r="B6" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A6,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A6,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>11.5</v>
       </c>
       <c r="C6" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A6,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A6,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>632.5</v>
       </c>
       <c r="D6" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A6,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A6,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>7.61</v>
       </c>
       <c r="E6" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A6,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A6,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>91.32</v>
       </c>
       <c r="F6" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A6,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A6,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>53.9</v>
       </c>
       <c r="G6" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A6,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A6,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>835.45</v>
       </c>
       <c r="H6" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A6,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A6,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1</v>
       </c>
       <c r="I6" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A6,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A6,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1032</v>
       </c>
       <c r="J6" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A6,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A6,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K6" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A6,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A6,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L6" s="10" t="n">
@@ -1265,43 +1280,43 @@
         <v>16</v>
       </c>
       <c r="B7" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A7,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A7,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>11.75</v>
       </c>
       <c r="C7" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A7,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A7,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>646.25</v>
       </c>
       <c r="D7" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A7,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A7,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>6.66</v>
       </c>
       <c r="E7" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A7,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A7,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>79.92</v>
       </c>
       <c r="F7" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A7,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A7,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>53.9</v>
       </c>
       <c r="G7" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A7,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A7,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>835.45</v>
       </c>
       <c r="H7" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A7,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A7,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1</v>
       </c>
       <c r="I7" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A7,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A7,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1032</v>
       </c>
       <c r="J7" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A7,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A7,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K7" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A7,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A7,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L7" s="10" t="n">
@@ -1314,43 +1329,43 @@
         <v>17</v>
       </c>
       <c r="B8" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A8,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A8,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="C8" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A8,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A8,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="D8" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A8,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A8,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>18.235</v>
       </c>
       <c r="E8" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A8,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A8,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>218.82</v>
       </c>
       <c r="F8" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A8,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A8,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>53.9</v>
       </c>
       <c r="G8" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A8,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A8,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>835.45</v>
       </c>
       <c r="H8" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A8,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A8,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1</v>
       </c>
       <c r="I8" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A8,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A8,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1032</v>
       </c>
       <c r="J8" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A8,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A8,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K8" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A8,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A8,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L8" s="10" t="n">
@@ -1363,43 +1378,43 @@
         <v>18</v>
       </c>
       <c r="B9" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A9,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A9,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>10.375</v>
       </c>
       <c r="C9" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A9,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A9,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>570.625</v>
       </c>
       <c r="D9" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A9,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A9,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>41.985</v>
       </c>
       <c r="E9" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A9,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A9,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>503.82</v>
       </c>
       <c r="F9" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A9,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A9,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>50.4</v>
       </c>
       <c r="G9" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A9,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A9,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>781.2</v>
       </c>
       <c r="H9" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A9,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A9,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1</v>
       </c>
       <c r="I9" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A9,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A9,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1032</v>
       </c>
       <c r="J9" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A9,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A9,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K9" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A9,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A9,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L9" s="10" t="n">
@@ -1412,43 +1427,43 @@
         <v>19</v>
       </c>
       <c r="B10" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A10,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A10,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="C10" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A10,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A10,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="D10" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A10,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A10,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>27.86</v>
       </c>
       <c r="E10" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A10,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A10,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>334.32</v>
       </c>
       <c r="F10" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A10,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A10,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>53.9</v>
       </c>
       <c r="G10" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A10,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A10,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>835.45</v>
       </c>
       <c r="H10" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A10,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A10,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1</v>
       </c>
       <c r="I10" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A10,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A10,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1032</v>
       </c>
       <c r="J10" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A10,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A10,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K10" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A10,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A10,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L10" s="10" t="n">
@@ -1461,43 +1476,43 @@
         <v>20</v>
       </c>
       <c r="B11" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A11,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A11,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>11.75</v>
       </c>
       <c r="C11" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A11,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A11,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>646.25</v>
       </c>
       <c r="D11" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A11,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A11,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>25.91</v>
       </c>
       <c r="E11" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A11,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A11,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>310.92</v>
       </c>
       <c r="F11" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A11,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A11,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>53.9</v>
       </c>
       <c r="G11" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A11,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A11,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>835.45</v>
       </c>
       <c r="H11" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A11,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A11,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1</v>
       </c>
       <c r="I11" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A11,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A11,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1032</v>
       </c>
       <c r="J11" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A11,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A11,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K11" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A11,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A11,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L11" s="10" t="n">
@@ -1510,43 +1525,43 @@
         <v>21</v>
       </c>
       <c r="B12" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A12,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A12,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>11.75</v>
       </c>
       <c r="C12" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A12,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A12,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>646.25</v>
       </c>
       <c r="D12" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A12,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A12,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>30.81</v>
       </c>
       <c r="E12" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A12,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A12,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>369.72</v>
       </c>
       <c r="F12" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A12,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A12,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>53.9</v>
       </c>
       <c r="G12" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A12,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A12,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>835.45</v>
       </c>
       <c r="H12" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A12,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A12,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1</v>
       </c>
       <c r="I12" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A12,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A12,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1032</v>
       </c>
       <c r="J12" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A12,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A12,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K12" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A12,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A12,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L12" s="10" t="n">
@@ -1559,48 +1574,48 @@
         <v>22</v>
       </c>
       <c r="B13" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A13,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A13,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="C13" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A13,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A13,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="D13" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A13,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A13,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>0</v>
       </c>
       <c r="E13" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A13,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A13,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>0</v>
       </c>
       <c r="F13" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A13,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
-        <v>0</v>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A13,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
+        <v>46.86</v>
       </c>
       <c r="G13" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A13,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
-        <v>0</v>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A13,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
+        <v>726.33</v>
       </c>
       <c r="H13" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A13,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A13,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1</v>
       </c>
       <c r="I13" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A13,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A13,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>1032</v>
       </c>
       <c r="J13" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A13,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A13,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K13" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A13,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A13,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L13" s="10" t="n">
         <f aca="false">C13+E13+G13+I13+K13</f>
-        <v>1032</v>
+        <v>1758.33</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1625,11 +1640,11 @@
       </c>
       <c r="F14" s="12" t="n">
         <f aca="false">SUM(F6:F13)</f>
-        <v>373.8</v>
+        <v>420.66</v>
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">SUM(G6:G13)</f>
-        <v>5793.9</v>
+        <v>6520.23</v>
       </c>
       <c r="H14" s="14" t="n">
         <f aca="false">SUM(H6:H13)</f>
@@ -1649,7 +1664,7 @@
       </c>
       <c r="L14" s="13" t="n">
         <f aca="false">SUM(L6:L13)</f>
-        <v>19100.615</v>
+        <v>19826.945</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1673,43 +1688,43 @@
         <v>25</v>
       </c>
       <c r="B17" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A17,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A17,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>4.75</v>
       </c>
       <c r="C17" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A17,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A17,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>261.25</v>
       </c>
       <c r="D17" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A17,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A17,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>34.66</v>
       </c>
       <c r="E17" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A17,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A17,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>415.92</v>
       </c>
       <c r="F17" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A17,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A17,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>39.2</v>
       </c>
       <c r="G17" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A17,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A17,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>607.6</v>
       </c>
       <c r="H17" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A17,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A17,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="I17" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A17,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A17,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="J17" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A17,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A17,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K17" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A17,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A17,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L17" s="10" t="n">
@@ -1722,43 +1737,43 @@
         <v>26</v>
       </c>
       <c r="B18" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A18,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A18,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>4.75</v>
       </c>
       <c r="C18" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A18,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A18,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>261.25</v>
       </c>
       <c r="D18" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A18,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A18,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>35.71</v>
       </c>
       <c r="E18" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A18,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A18,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>428.52</v>
       </c>
       <c r="F18" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A18,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A18,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>39.2</v>
       </c>
       <c r="G18" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A18,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A18,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>607.6</v>
       </c>
       <c r="H18" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A18,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A18,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="I18" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A18,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A18,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="J18" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A18,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A18,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K18" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A18,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A18,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L18" s="10" t="n">
@@ -1771,43 +1786,43 @@
         <v>27</v>
       </c>
       <c r="B19" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A19,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A19,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="C19" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A19,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A19,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="D19" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A19,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A19,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>40.81</v>
       </c>
       <c r="E19" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A19,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A19,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>489.72</v>
       </c>
       <c r="F19" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A19,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A19,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>39.2</v>
       </c>
       <c r="G19" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A19,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A19,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>607.6</v>
       </c>
       <c r="H19" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A19,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A19,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="I19" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A19,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A19,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="J19" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A19,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A19,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K19" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A19,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A19,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L19" s="10" t="n">
@@ -1820,43 +1835,43 @@
         <v>28</v>
       </c>
       <c r="B20" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A20,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A20,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="C20" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A20,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A20,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="D20" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A20,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A20,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>41.16</v>
       </c>
       <c r="E20" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A20,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A20,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>493.92</v>
       </c>
       <c r="F20" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A20,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A20,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>39.2</v>
       </c>
       <c r="G20" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A20,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A20,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>607.6</v>
       </c>
       <c r="H20" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A20,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A20,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="I20" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A20,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A20,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="J20" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A20,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A20,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K20" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A20,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A20,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L20" s="10" t="n">
@@ -1869,43 +1884,43 @@
         <v>29</v>
       </c>
       <c r="B21" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A21,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A21,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="C21" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A21,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A21,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="D21" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A21,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A21,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>0</v>
       </c>
       <c r="E21" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A21,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A21,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>0</v>
       </c>
       <c r="F21" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A21,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A21,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>29.26</v>
       </c>
       <c r="G21" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A21,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A21,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>453.53</v>
       </c>
       <c r="H21" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A21,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A21,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="I21" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A21,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A21,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="J21" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A21,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A21,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K21" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A21,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A21,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L21" s="10" t="n">
@@ -1983,43 +1998,43 @@
         <v>32</v>
       </c>
       <c r="B25" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A25,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A25,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="C25" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A25,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A25,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="D25" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A25,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A25,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>57.275</v>
       </c>
       <c r="E25" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A25,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A25,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>687.3</v>
       </c>
       <c r="F25" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A25,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A25,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>0</v>
       </c>
       <c r="G25" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A25,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A25,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>0</v>
       </c>
       <c r="H25" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A25,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A25,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="I25" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A25,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A25,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="J25" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A25,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A25,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K25" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A25,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A25,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L25" s="10" t="n">
@@ -2032,43 +2047,43 @@
         <v>33</v>
       </c>
       <c r="B26" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A26,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A26,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="C26" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A26,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A26,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="D26" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A26,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A26,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>48.51</v>
       </c>
       <c r="E26" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A26,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A26,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>582.12</v>
       </c>
       <c r="F26" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A26,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A26,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>0</v>
       </c>
       <c r="G26" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A26,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A26,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>0</v>
       </c>
       <c r="H26" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A26,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A26,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="I26" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A26,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A26,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="J26" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A26,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A26,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K26" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A26,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A26,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L26" s="10" t="n">
@@ -2081,43 +2096,43 @@
         <v>34</v>
       </c>
       <c r="B27" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A27,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A27,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="C27" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A27,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A27,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="D27" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A27,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A27,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>9.625</v>
       </c>
       <c r="E27" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A27,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A27,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>115.5</v>
       </c>
       <c r="F27" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A27,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A27,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>0</v>
       </c>
       <c r="G27" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A27,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A27,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>0</v>
       </c>
       <c r="H27" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A27,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A27,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="I27" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A27,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A27,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="J27" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A27,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A27,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K27" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A27,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A27,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L27" s="10" t="n">
@@ -2130,43 +2145,43 @@
         <v>35</v>
       </c>
       <c r="B28" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A28,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A28,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="C28" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A28,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A28,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="D28" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A28,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A28,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>9.1</v>
       </c>
       <c r="E28" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A28,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A28,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>109.2</v>
       </c>
       <c r="F28" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A28,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A28,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>0</v>
       </c>
       <c r="G28" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A28,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A28,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>0</v>
       </c>
       <c r="H28" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A28,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A28,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="I28" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A28,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A28,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="J28" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A28,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A28,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="K28" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A28,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A28,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>0</v>
       </c>
       <c r="L28" s="10" t="n">
@@ -2179,43 +2194,43 @@
         <v>36</v>
       </c>
       <c r="B29" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A29,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A29,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="C29" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A29,'Hisob (batafsil)'!$C$5:$C$200,"Shisha devor")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A29,'Hisob (batafsil)'!$C$5:$C$204,"Shisha devor")</f>
         <v>0</v>
       </c>
       <c r="D29" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A29,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A29,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>0</v>
       </c>
       <c r="E29" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A29,'Hisob (batafsil)'!$C$5:$C$200,"Gips karton (GKL)")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A29,'Hisob (batafsil)'!$C$5:$C$204,"Gips karton (GKL)")</f>
         <v>0</v>
       </c>
       <c r="F29" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A29,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A29,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>0</v>
       </c>
       <c r="G29" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A29,'Hisob (batafsil)'!$C$5:$C$200,"Bambuk panel")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A29,'Hisob (batafsil)'!$C$5:$C$204,"Bambuk panel")</f>
         <v>0</v>
       </c>
       <c r="H29" s="9" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A29,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A29,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="I29" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A29,'Hisob (batafsil)'!$C$5:$C$200,"Interaktiv doska")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A29,'Hisob (batafsil)'!$C$5:$C$204,"Interaktiv doska")</f>
         <v>0</v>
       </c>
       <c r="J29" s="7" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$200,'Hisob (batafsil)'!$B$5:$B$200,$A29,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$G$5:$G$204,'Hisob (batafsil)'!$B$5:$B$204,$A29,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>24</v>
       </c>
       <c r="K29" s="8" t="n">
-        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$200,'Hisob (batafsil)'!$B$5:$B$200,$A29,'Hisob (batafsil)'!$C$5:$C$200,"Perila")</f>
+        <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$204,'Hisob (batafsil)'!$B$5:$B$204,$A29,'Hisob (batafsil)'!$C$5:$C$204,"Perila")</f>
         <v>2016</v>
       </c>
       <c r="L29" s="10" t="n">
@@ -2294,11 +2309,11 @@
       </c>
       <c r="F32" s="16" t="n">
         <f aca="false">F14+F22+F30</f>
-        <v>559.86</v>
+        <v>606.72</v>
       </c>
       <c r="G32" s="17" t="n">
         <f aca="false">G14+G22+G30</f>
-        <v>8677.83</v>
+        <v>9404.16</v>
       </c>
       <c r="H32" s="18" t="n">
         <f aca="false">H14+H22+H30</f>
@@ -2318,7 +2333,7 @@
       </c>
       <c r="L32" s="17" t="n">
         <f aca="false">L14+L22+L30</f>
-        <v>27845.245</v>
+        <v>28571.575</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2326,7 +2341,7 @@
         <v>39</v>
       </c>
       <c r="L34" s="19" t="n">
-        <f aca="false">L32-'Hisob (batafsil)'!J201</f>
+        <f aca="false">L32-'Hisob (batafsil)'!J205</f>
         <v>0</v>
       </c>
     </row>
@@ -2346,7 +2361,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2607,13 +2622,25 @@
         <v>72</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="25" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>73</v>
       </c>
+      <c r="C18" s="22" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="25" t="s">
         <v>74</v>
       </c>
     </row>
@@ -2655,6 +2682,16 @@
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
         <v>82</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -2673,7 +2710,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J201"/>
+  <dimension ref="A1:J205"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2689,12 +2726,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2705,28 +2742,28 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>45</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2754,7 +2791,7 @@
         <v>47</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>4.6</v>
@@ -2768,7 +2805,7 @@
         <v>11.5</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I6" s="28" t="n">
         <f aca="false">Narxlar!$C$5</f>
@@ -2787,10 +2824,10 @@
         <v>15</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E7" s="26" t="n">
         <v>0.3</v>
@@ -2804,7 +2841,7 @@
         <v>1.05</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I7" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -2823,10 +2860,10 @@
         <v>15</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>4.6</v>
@@ -2840,7 +2877,7 @@
         <v>4.6</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I8" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -2859,10 +2896,10 @@
         <v>15</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E9" s="26" t="n">
         <v>0.2</v>
@@ -2876,7 +2913,7 @@
         <v>0.7</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I9" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -2895,10 +2932,10 @@
         <v>15</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E10" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -2913,7 +2950,7 @@
         <v>1.26</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I10" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -2935,7 +2972,7 @@
         <v>52</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E11" s="26" t="n">
         <v>7.7</v>
@@ -2949,7 +2986,7 @@
         <v>26.95</v>
       </c>
       <c r="H11" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I11" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -2971,7 +3008,7 @@
         <v>52</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>7.7</v>
@@ -2985,7 +3022,7 @@
         <v>26.95</v>
       </c>
       <c r="H12" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I12" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -3007,7 +3044,7 @@
         <v>53</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E13" s="26"/>
       <c r="F13" s="27"/>
@@ -3015,7 +3052,7 @@
         <v>1</v>
       </c>
       <c r="H13" s="20" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I13" s="28" t="n">
         <f aca="false">Narxlar!$C$8</f>
@@ -3031,7 +3068,7 @@
       <c r="B14" s="31"/>
       <c r="C14" s="31"/>
       <c r="D14" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E14" s="31"/>
       <c r="F14" s="31"/>
@@ -3068,7 +3105,7 @@
         <v>47</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E17" s="26" t="n">
         <v>4.7</v>
@@ -3082,7 +3119,7 @@
         <v>11.75</v>
       </c>
       <c r="H17" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I17" s="28" t="n">
         <f aca="false">Narxlar!$C$5</f>
@@ -3101,10 +3138,10 @@
         <v>16</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E18" s="26" t="n">
         <v>4.7</v>
@@ -3118,7 +3155,7 @@
         <v>4.7</v>
       </c>
       <c r="H18" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I18" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3137,10 +3174,10 @@
         <v>16</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E19" s="26" t="n">
         <v>0.2</v>
@@ -3154,7 +3191,7 @@
         <v>0.7</v>
       </c>
       <c r="H19" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I19" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3173,10 +3210,10 @@
         <v>16</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E20" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -3191,7 +3228,7 @@
         <v>1.26</v>
       </c>
       <c r="H20" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I20" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3213,7 +3250,7 @@
         <v>52</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E21" s="26" t="n">
         <v>7.7</v>
@@ -3227,7 +3264,7 @@
         <v>26.95</v>
       </c>
       <c r="H21" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I21" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -3249,7 +3286,7 @@
         <v>52</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E22" s="26" t="n">
         <v>7.7</v>
@@ -3263,7 +3300,7 @@
         <v>26.95</v>
       </c>
       <c r="H22" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I22" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -3285,7 +3322,7 @@
         <v>53</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E23" s="26"/>
       <c r="F23" s="27"/>
@@ -3293,7 +3330,7 @@
         <v>1</v>
       </c>
       <c r="H23" s="20" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I23" s="28" t="n">
         <f aca="false">Narxlar!$C$8</f>
@@ -3309,7 +3346,7 @@
       <c r="B24" s="31"/>
       <c r="C24" s="31"/>
       <c r="D24" s="11" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -3343,10 +3380,10 @@
         <v>17</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E27" s="26" t="n">
         <v>0.15</v>
@@ -3360,7 +3397,7 @@
         <v>0.525</v>
       </c>
       <c r="H27" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I27" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3379,10 +3416,10 @@
         <v>17</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E28" s="26" t="n">
         <v>4.7</v>
@@ -3396,7 +3433,7 @@
         <v>16.45</v>
       </c>
       <c r="H28" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I28" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3415,10 +3452,10 @@
         <v>17</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E29" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -3433,7 +3470,7 @@
         <v>1.26</v>
       </c>
       <c r="H29" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I29" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3455,7 +3492,7 @@
         <v>52</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E30" s="26" t="n">
         <v>7.7</v>
@@ -3469,7 +3506,7 @@
         <v>26.95</v>
       </c>
       <c r="H30" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I30" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -3491,7 +3528,7 @@
         <v>52</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E31" s="26" t="n">
         <v>7.7</v>
@@ -3505,7 +3542,7 @@
         <v>26.95</v>
       </c>
       <c r="H31" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I31" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -3527,7 +3564,7 @@
         <v>53</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E32" s="26"/>
       <c r="F32" s="27"/>
@@ -3535,7 +3572,7 @@
         <v>1</v>
       </c>
       <c r="H32" s="20" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I32" s="28" t="n">
         <f aca="false">Narxlar!$C$8</f>
@@ -3551,7 +3588,7 @@
       <c r="B33" s="31"/>
       <c r="C33" s="31"/>
       <c r="D33" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E33" s="31"/>
       <c r="F33" s="31"/>
@@ -3588,7 +3625,7 @@
         <v>47</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E36" s="26" t="n">
         <v>1.5</v>
@@ -3602,7 +3639,7 @@
         <v>3.75</v>
       </c>
       <c r="H36" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I36" s="28" t="n">
         <f aca="false">Narxlar!$C$5</f>
@@ -3624,7 +3661,7 @@
         <v>47</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E37" s="26" t="n">
         <v>1.15</v>
@@ -3638,7 +3675,7 @@
         <v>2.875</v>
       </c>
       <c r="H37" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I37" s="28" t="n">
         <f aca="false">Narxlar!$C$5</f>
@@ -3660,7 +3697,7 @@
         <v>47</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E38" s="26" t="n">
         <v>1.5</v>
@@ -3674,7 +3711,7 @@
         <v>3.75</v>
       </c>
       <c r="H38" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I38" s="28" t="n">
         <f aca="false">Narxlar!$C$5</f>
@@ -3693,10 +3730,10 @@
         <v>18</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E39" s="26" t="n">
         <v>1</v>
@@ -3710,7 +3747,7 @@
         <v>3.5</v>
       </c>
       <c r="H39" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I39" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3729,10 +3766,10 @@
         <v>18</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E40" s="26" t="n">
         <v>4.5</v>
@@ -3746,7 +3783,7 @@
         <v>15.75</v>
       </c>
       <c r="H40" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I40" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3765,10 +3802,10 @@
         <v>18</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E41" s="26" t="n">
         <v>1.5</v>
@@ -3782,7 +3819,7 @@
         <v>1.5</v>
       </c>
       <c r="H41" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I41" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3801,10 +3838,10 @@
         <v>18</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E42" s="26" t="n">
         <v>1.15</v>
@@ -3818,7 +3855,7 @@
         <v>1.15</v>
       </c>
       <c r="H42" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I42" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3837,10 +3874,10 @@
         <v>18</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E43" s="26" t="n">
         <v>0.1</v>
@@ -3854,7 +3891,7 @@
         <v>0.35</v>
       </c>
       <c r="H43" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I43" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3873,10 +3910,10 @@
         <v>18</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E44" s="26" t="n">
         <v>0.1</v>
@@ -3890,7 +3927,7 @@
         <v>0.35</v>
       </c>
       <c r="H44" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I44" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3909,10 +3946,10 @@
         <v>18</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E45" s="26" t="n">
         <v>0.25</v>
@@ -3926,7 +3963,7 @@
         <v>0.875</v>
       </c>
       <c r="H45" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I45" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3945,10 +3982,10 @@
         <v>18</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E46" s="26" t="n">
         <v>1.5</v>
@@ -3962,7 +3999,7 @@
         <v>1.5</v>
       </c>
       <c r="H46" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I46" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -3981,10 +4018,10 @@
         <v>18</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E47" s="26" t="n">
         <v>4.5</v>
@@ -3998,7 +4035,7 @@
         <v>15.75</v>
       </c>
       <c r="H47" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I47" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4017,10 +4054,10 @@
         <v>18</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E48" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -4035,7 +4072,7 @@
         <v>1.26</v>
       </c>
       <c r="H48" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I48" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4057,7 +4094,7 @@
         <v>52</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E49" s="26" t="n">
         <v>8.8</v>
@@ -4071,7 +4108,7 @@
         <v>30.8</v>
       </c>
       <c r="H49" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I49" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -4093,7 +4130,7 @@
         <v>52</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E50" s="26" t="n">
         <v>5.6</v>
@@ -4107,7 +4144,7 @@
         <v>19.6</v>
       </c>
       <c r="H50" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I50" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -4129,7 +4166,7 @@
         <v>53</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E51" s="26"/>
       <c r="F51" s="27"/>
@@ -4137,7 +4174,7 @@
         <v>1</v>
       </c>
       <c r="H51" s="20" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I51" s="28" t="n">
         <f aca="false">Narxlar!$C$8</f>
@@ -4153,7 +4190,7 @@
       <c r="B52" s="31"/>
       <c r="C52" s="31"/>
       <c r="D52" s="11" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E52" s="31"/>
       <c r="F52" s="31"/>
@@ -4187,10 +4224,10 @@
         <v>19</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E55" s="26" t="n">
         <v>2.75</v>
@@ -4204,7 +4241,7 @@
         <v>9.625</v>
       </c>
       <c r="H55" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I55" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4223,10 +4260,10 @@
         <v>19</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E56" s="26" t="n">
         <v>0.15</v>
@@ -4240,7 +4277,7 @@
         <v>0.525</v>
       </c>
       <c r="H56" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I56" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4259,10 +4296,10 @@
         <v>19</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E57" s="26" t="n">
         <v>4.7</v>
@@ -4276,7 +4313,7 @@
         <v>16.45</v>
       </c>
       <c r="H57" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I57" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4295,10 +4332,10 @@
         <v>19</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E58" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -4313,7 +4350,7 @@
         <v>1.26</v>
       </c>
       <c r="H58" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I58" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4335,7 +4372,7 @@
         <v>52</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E59" s="26" t="n">
         <v>7.7</v>
@@ -4349,7 +4386,7 @@
         <v>26.95</v>
       </c>
       <c r="H59" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I59" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -4371,7 +4408,7 @@
         <v>52</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E60" s="26" t="n">
         <v>7.7</v>
@@ -4385,7 +4422,7 @@
         <v>26.95</v>
       </c>
       <c r="H60" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I60" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -4407,7 +4444,7 @@
         <v>53</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E61" s="26"/>
       <c r="F61" s="27"/>
@@ -4415,7 +4452,7 @@
         <v>1</v>
       </c>
       <c r="H61" s="20" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I61" s="28" t="n">
         <f aca="false">Narxlar!$C$8</f>
@@ -4431,7 +4468,7 @@
       <c r="B62" s="31"/>
       <c r="C62" s="31"/>
       <c r="D62" s="11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E62" s="31"/>
       <c r="F62" s="31"/>
@@ -4468,7 +4505,7 @@
         <v>47</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E65" s="26" t="n">
         <v>4.7</v>
@@ -4482,7 +4519,7 @@
         <v>11.75</v>
       </c>
       <c r="H65" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I65" s="28" t="n">
         <f aca="false">Narxlar!$C$5</f>
@@ -4501,10 +4538,10 @@
         <v>20</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E66" s="26" t="n">
         <v>2.75</v>
@@ -4518,7 +4555,7 @@
         <v>9.625</v>
       </c>
       <c r="H66" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I66" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4537,10 +4574,10 @@
         <v>20</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E67" s="26" t="n">
         <v>2.75</v>
@@ -4554,7 +4591,7 @@
         <v>9.625</v>
       </c>
       <c r="H67" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I67" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4573,10 +4610,10 @@
         <v>20</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E68" s="26" t="n">
         <v>0.2</v>
@@ -4590,7 +4627,7 @@
         <v>0.7</v>
       </c>
       <c r="H68" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I68" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4609,10 +4646,10 @@
         <v>20</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E69" s="26" t="n">
         <v>4.7</v>
@@ -4626,7 +4663,7 @@
         <v>4.7</v>
       </c>
       <c r="H69" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I69" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4645,10 +4682,10 @@
         <v>20</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E70" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -4663,7 +4700,7 @@
         <v>1.26</v>
       </c>
       <c r="H70" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I70" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4685,7 +4722,7 @@
         <v>52</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E71" s="26" t="n">
         <v>7.7</v>
@@ -4699,7 +4736,7 @@
         <v>26.95</v>
       </c>
       <c r="H71" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I71" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -4721,7 +4758,7 @@
         <v>52</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E72" s="26" t="n">
         <v>7.7</v>
@@ -4735,7 +4772,7 @@
         <v>26.95</v>
       </c>
       <c r="H72" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I72" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -4757,7 +4794,7 @@
         <v>53</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E73" s="26"/>
       <c r="F73" s="27"/>
@@ -4765,7 +4802,7 @@
         <v>1</v>
       </c>
       <c r="H73" s="20" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I73" s="28" t="n">
         <f aca="false">Narxlar!$C$8</f>
@@ -4781,7 +4818,7 @@
       <c r="B74" s="31"/>
       <c r="C74" s="31"/>
       <c r="D74" s="11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E74" s="31"/>
       <c r="F74" s="31"/>
@@ -4818,7 +4855,7 @@
         <v>47</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E77" s="26" t="n">
         <v>4.7</v>
@@ -4832,7 +4869,7 @@
         <v>11.75</v>
       </c>
       <c r="H77" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I77" s="28" t="n">
         <f aca="false">Narxlar!$C$5</f>
@@ -4851,10 +4888,10 @@
         <v>21</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E78" s="26" t="n">
         <v>1.55</v>
@@ -4868,7 +4905,7 @@
         <v>5.425</v>
       </c>
       <c r="H78" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I78" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4887,10 +4924,10 @@
         <v>21</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E79" s="26" t="n">
         <v>2.6</v>
@@ -4904,7 +4941,7 @@
         <v>9.1</v>
       </c>
       <c r="H79" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I79" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4923,10 +4960,10 @@
         <v>21</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E80" s="26" t="n">
         <v>2.75</v>
@@ -4940,7 +4977,7 @@
         <v>9.625</v>
       </c>
       <c r="H80" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I80" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4959,10 +4996,10 @@
         <v>21</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E81" s="26" t="n">
         <v>0.2</v>
@@ -4976,7 +5013,7 @@
         <v>0.7</v>
       </c>
       <c r="H81" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I81" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -4995,10 +5032,10 @@
         <v>21</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E82" s="26" t="n">
         <v>4.7</v>
@@ -5012,7 +5049,7 @@
         <v>4.7</v>
       </c>
       <c r="H82" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I82" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5031,10 +5068,10 @@
         <v>21</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E83" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -5049,7 +5086,7 @@
         <v>1.26</v>
       </c>
       <c r="H83" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I83" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5071,7 +5108,7 @@
         <v>52</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E84" s="26" t="n">
         <v>7.7</v>
@@ -5085,7 +5122,7 @@
         <v>26.95</v>
       </c>
       <c r="H84" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I84" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -5107,7 +5144,7 @@
         <v>52</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E85" s="26" t="n">
         <v>7.7</v>
@@ -5121,7 +5158,7 @@
         <v>26.95</v>
       </c>
       <c r="H85" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I85" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -5143,7 +5180,7 @@
         <v>53</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E86" s="26"/>
       <c r="F86" s="27"/>
@@ -5151,7 +5188,7 @@
         <v>1</v>
       </c>
       <c r="H86" s="20" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I86" s="28" t="n">
         <f aca="false">Narxlar!$C$8</f>
@@ -5167,7 +5204,7 @@
       <c r="B87" s="31"/>
       <c r="C87" s="31"/>
       <c r="D87" s="11" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E87" s="31"/>
       <c r="F87" s="31"/>
@@ -5204,7 +5241,7 @@
         <v>47</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E90" s="26" t="n">
         <v>0.15</v>
@@ -5218,7 +5255,7 @@
         <v>0.375</v>
       </c>
       <c r="H90" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I90" s="28" t="n">
         <f aca="false">Narxlar!$C$5</f>
@@ -5240,7 +5277,7 @@
         <v>47</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E91" s="26" t="n">
         <v>1.75</v>
@@ -5254,7 +5291,7 @@
         <v>4.375</v>
       </c>
       <c r="H91" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I91" s="28" t="n">
         <f aca="false">Narxlar!$C$5</f>
@@ -5273,10 +5310,10 @@
         <v>25</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E92" s="26" t="n">
         <v>0.6</v>
@@ -5290,7 +5327,7 @@
         <v>2.1</v>
       </c>
       <c r="H92" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I92" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5309,10 +5346,10 @@
         <v>25</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E93" s="26" t="n">
         <v>2.8</v>
@@ -5326,7 +5363,7 @@
         <v>9.8</v>
       </c>
       <c r="H93" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I93" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5345,10 +5382,10 @@
         <v>25</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E94" s="26" t="n">
         <v>5.6</v>
@@ -5362,7 +5399,7 @@
         <v>19.6</v>
       </c>
       <c r="H94" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I94" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5381,10 +5418,10 @@
         <v>25</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E95" s="26" t="n">
         <v>0.15</v>
@@ -5398,7 +5435,7 @@
         <v>0.15</v>
       </c>
       <c r="H95" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I95" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5417,10 +5454,10 @@
         <v>25</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E96" s="26" t="n">
         <v>1.75</v>
@@ -5434,7 +5471,7 @@
         <v>1.75</v>
       </c>
       <c r="H96" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I96" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5453,10 +5490,10 @@
         <v>25</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D97" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E97" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -5471,7 +5508,7 @@
         <v>1.26</v>
       </c>
       <c r="H97" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I97" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5493,7 +5530,7 @@
         <v>52</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E98" s="26" t="n">
         <v>5.6</v>
@@ -5507,7 +5544,7 @@
         <v>19.6</v>
       </c>
       <c r="H98" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I98" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -5529,7 +5566,7 @@
         <v>52</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E99" s="26" t="n">
         <v>5.6</v>
@@ -5543,7 +5580,7 @@
         <v>19.6</v>
       </c>
       <c r="H99" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I99" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -5559,7 +5596,7 @@
       <c r="B100" s="31"/>
       <c r="C100" s="31"/>
       <c r="D100" s="11" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E100" s="31"/>
       <c r="F100" s="31"/>
@@ -5596,7 +5633,7 @@
         <v>47</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E103" s="26" t="n">
         <v>0.15</v>
@@ -5610,7 +5647,7 @@
         <v>0.375</v>
       </c>
       <c r="H103" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I103" s="28" t="n">
         <f aca="false">Narxlar!$C$5</f>
@@ -5632,7 +5669,7 @@
         <v>47</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E104" s="26" t="n">
         <v>1.75</v>
@@ -5646,7 +5683,7 @@
         <v>4.375</v>
       </c>
       <c r="H104" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I104" s="28" t="n">
         <f aca="false">Narxlar!$C$5</f>
@@ -5665,10 +5702,10 @@
         <v>26</v>
       </c>
       <c r="C105" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E105" s="26" t="n">
         <v>0.9</v>
@@ -5682,7 +5719,7 @@
         <v>3.15</v>
       </c>
       <c r="H105" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I105" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5701,10 +5738,10 @@
         <v>26</v>
       </c>
       <c r="C106" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E106" s="26" t="n">
         <v>2.8</v>
@@ -5718,7 +5755,7 @@
         <v>9.8</v>
       </c>
       <c r="H106" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I106" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5737,10 +5774,10 @@
         <v>26</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E107" s="26" t="n">
         <v>5.6</v>
@@ -5754,7 +5791,7 @@
         <v>19.6</v>
       </c>
       <c r="H107" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I107" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5773,10 +5810,10 @@
         <v>26</v>
       </c>
       <c r="C108" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E108" s="26" t="n">
         <v>0.15</v>
@@ -5790,7 +5827,7 @@
         <v>0.15</v>
       </c>
       <c r="H108" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I108" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5809,10 +5846,10 @@
         <v>26</v>
       </c>
       <c r="C109" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D109" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E109" s="26" t="n">
         <v>1.75</v>
@@ -5826,7 +5863,7 @@
         <v>1.75</v>
       </c>
       <c r="H109" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I109" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5845,10 +5882,10 @@
         <v>26</v>
       </c>
       <c r="C110" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D110" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E110" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -5863,7 +5900,7 @@
         <v>1.26</v>
       </c>
       <c r="H110" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I110" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -5885,7 +5922,7 @@
         <v>52</v>
       </c>
       <c r="D111" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E111" s="26" t="n">
         <v>5.6</v>
@@ -5899,7 +5936,7 @@
         <v>19.6</v>
       </c>
       <c r="H111" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I111" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -5921,7 +5958,7 @@
         <v>52</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E112" s="26" t="n">
         <v>5.6</v>
@@ -5935,7 +5972,7 @@
         <v>19.6</v>
       </c>
       <c r="H112" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I112" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -5951,7 +5988,7 @@
       <c r="B113" s="31"/>
       <c r="C113" s="31"/>
       <c r="D113" s="11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E113" s="31"/>
       <c r="F113" s="31"/>
@@ -5985,10 +6022,10 @@
         <v>27</v>
       </c>
       <c r="C116" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E116" s="26" t="n">
         <v>0.9</v>
@@ -6002,7 +6039,7 @@
         <v>3.15</v>
       </c>
       <c r="H116" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I116" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6021,10 +6058,10 @@
         <v>27</v>
       </c>
       <c r="C117" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E117" s="26" t="n">
         <v>0.15</v>
@@ -6038,7 +6075,7 @@
         <v>0.525</v>
       </c>
       <c r="H117" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I117" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6057,10 +6094,10 @@
         <v>27</v>
       </c>
       <c r="C118" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E118" s="26" t="n">
         <v>1.8</v>
@@ -6074,7 +6111,7 @@
         <v>6.3</v>
       </c>
       <c r="H118" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I118" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6093,10 +6130,10 @@
         <v>27</v>
       </c>
       <c r="C119" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D119" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E119" s="26" t="n">
         <v>5.6</v>
@@ -6110,7 +6147,7 @@
         <v>19.6</v>
       </c>
       <c r="H119" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I119" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6129,10 +6166,10 @@
         <v>27</v>
       </c>
       <c r="C120" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D120" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E120" s="26" t="n">
         <v>2.85</v>
@@ -6146,7 +6183,7 @@
         <v>9.975</v>
       </c>
       <c r="H120" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I120" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6165,10 +6202,10 @@
         <v>27</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D121" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E121" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -6183,7 +6220,7 @@
         <v>1.26</v>
       </c>
       <c r="H121" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I121" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6205,7 +6242,7 @@
         <v>52</v>
       </c>
       <c r="D122" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E122" s="26" t="n">
         <v>5.6</v>
@@ -6219,7 +6256,7 @@
         <v>19.6</v>
       </c>
       <c r="H122" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I122" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -6241,7 +6278,7 @@
         <v>52</v>
       </c>
       <c r="D123" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E123" s="26" t="n">
         <v>5.6</v>
@@ -6255,7 +6292,7 @@
         <v>19.6</v>
       </c>
       <c r="H123" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I123" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -6271,7 +6308,7 @@
       <c r="B124" s="31"/>
       <c r="C124" s="31"/>
       <c r="D124" s="11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E124" s="31"/>
       <c r="F124" s="31"/>
@@ -6305,10 +6342,10 @@
         <v>28</v>
       </c>
       <c r="C127" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D127" s="6" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E127" s="26" t="n">
         <v>1</v>
@@ -6322,7 +6359,7 @@
         <v>3.5</v>
       </c>
       <c r="H127" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I127" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6341,10 +6378,10 @@
         <v>28</v>
       </c>
       <c r="C128" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D128" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E128" s="26" t="n">
         <v>0.15</v>
@@ -6358,7 +6395,7 @@
         <v>0.525</v>
       </c>
       <c r="H128" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I128" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6377,10 +6414,10 @@
         <v>28</v>
       </c>
       <c r="C129" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D129" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E129" s="26" t="n">
         <v>1.8</v>
@@ -6394,7 +6431,7 @@
         <v>6.3</v>
       </c>
       <c r="H129" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I129" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6413,10 +6450,10 @@
         <v>28</v>
       </c>
       <c r="C130" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D130" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E130" s="26" t="n">
         <v>5.6</v>
@@ -6430,7 +6467,7 @@
         <v>19.6</v>
       </c>
       <c r="H130" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I130" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6449,10 +6486,10 @@
         <v>28</v>
       </c>
       <c r="C131" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D131" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E131" s="26" t="n">
         <v>2.85</v>
@@ -6466,7 +6503,7 @@
         <v>9.975</v>
       </c>
       <c r="H131" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I131" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6485,10 +6522,10 @@
         <v>28</v>
       </c>
       <c r="C132" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D132" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E132" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -6503,7 +6540,7 @@
         <v>1.26</v>
       </c>
       <c r="H132" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I132" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6525,7 +6562,7 @@
         <v>52</v>
       </c>
       <c r="D133" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E133" s="26" t="n">
         <v>5.6</v>
@@ -6539,7 +6576,7 @@
         <v>19.6</v>
       </c>
       <c r="H133" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I133" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -6561,7 +6598,7 @@
         <v>52</v>
       </c>
       <c r="D134" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E134" s="26" t="n">
         <v>5.6</v>
@@ -6575,7 +6612,7 @@
         <v>19.6</v>
       </c>
       <c r="H134" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I134" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -6591,7 +6628,7 @@
       <c r="B135" s="31"/>
       <c r="C135" s="31"/>
       <c r="D135" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E135" s="31"/>
       <c r="F135" s="31"/>
@@ -6628,7 +6665,7 @@
         <v>52</v>
       </c>
       <c r="D138" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E138" s="26" t="n">
         <v>5.95</v>
@@ -6642,7 +6679,7 @@
         <v>20.825</v>
       </c>
       <c r="H138" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I138" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -6664,7 +6701,7 @@
         <v>52</v>
       </c>
       <c r="D139" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E139" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -6679,7 +6716,7 @@
         <v>-1.89</v>
       </c>
       <c r="H139" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I139" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -6701,7 +6738,7 @@
         <v>52</v>
       </c>
       <c r="D140" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E140" s="26" t="n">
         <v>2.95</v>
@@ -6715,7 +6752,7 @@
         <v>10.325</v>
       </c>
       <c r="H140" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I140" s="28" t="n">
         <f aca="false">Narxlar!$C$7</f>
@@ -6731,7 +6768,7 @@
       <c r="B141" s="31"/>
       <c r="C141" s="31"/>
       <c r="D141" s="11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E141" s="31"/>
       <c r="F141" s="31"/>
@@ -6765,10 +6802,10 @@
         <v>32</v>
       </c>
       <c r="C144" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D144" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E144" s="26" t="n">
         <v>4.6</v>
@@ -6782,7 +6819,7 @@
         <v>4.6</v>
       </c>
       <c r="H144" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I144" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6801,10 +6838,10 @@
         <v>32</v>
       </c>
       <c r="C145" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D145" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E145" s="26" t="n">
         <v>0.4</v>
@@ -6818,7 +6855,7 @@
         <v>1.4</v>
       </c>
       <c r="H145" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I145" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6837,10 +6874,10 @@
         <v>32</v>
       </c>
       <c r="C146" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D146" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E146" s="26" t="n">
         <v>4.7</v>
@@ -6854,7 +6891,7 @@
         <v>4.7</v>
       </c>
       <c r="H146" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I146" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6873,10 +6910,10 @@
         <v>32</v>
       </c>
       <c r="C147" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D147" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E147" s="26" t="n">
         <v>0.55</v>
@@ -6890,7 +6927,7 @@
         <v>1.925</v>
       </c>
       <c r="H147" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I147" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6909,10 +6946,10 @@
         <v>32</v>
       </c>
       <c r="C148" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E148" s="26" t="n">
         <v>0.1</v>
@@ -6926,7 +6963,7 @@
         <v>0.35</v>
       </c>
       <c r="H148" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I148" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6945,10 +6982,10 @@
         <v>32</v>
       </c>
       <c r="C149" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D149" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E149" s="26" t="n">
         <v>1.5</v>
@@ -6962,7 +6999,7 @@
         <v>1.5</v>
       </c>
       <c r="H149" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I149" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -6981,10 +7018,10 @@
         <v>32</v>
       </c>
       <c r="C150" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D150" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E150" s="26" t="n">
         <v>6.05</v>
@@ -6998,7 +7035,7 @@
         <v>21.175</v>
       </c>
       <c r="H150" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I150" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7017,10 +7054,10 @@
         <v>32</v>
       </c>
       <c r="C151" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D151" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E151" s="26" t="n">
         <v>2.05</v>
@@ -7034,7 +7071,7 @@
         <v>7.175</v>
       </c>
       <c r="H151" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I151" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7053,10 +7090,10 @@
         <v>32</v>
       </c>
       <c r="C152" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D152" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E152" s="26" t="n">
         <v>2</v>
@@ -7070,7 +7107,7 @@
         <v>7</v>
       </c>
       <c r="H152" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I152" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7089,10 +7126,10 @@
         <v>32</v>
       </c>
       <c r="C153" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D153" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E153" s="26" t="n">
         <v>1.15</v>
@@ -7106,7 +7143,7 @@
         <v>1.15</v>
       </c>
       <c r="H153" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I153" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7125,10 +7162,10 @@
         <v>32</v>
       </c>
       <c r="C154" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D154" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E154" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -7143,7 +7180,7 @@
         <v>1.26</v>
       </c>
       <c r="H154" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I154" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7162,10 +7199,10 @@
         <v>32</v>
       </c>
       <c r="C155" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D155" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E155" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -7180,7 +7217,7 @@
         <v>1.26</v>
       </c>
       <c r="H155" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I155" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7199,10 +7236,10 @@
         <v>32</v>
       </c>
       <c r="C156" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D156" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E156" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -7217,7 +7254,7 @@
         <v>1.26</v>
       </c>
       <c r="H156" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I156" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7236,10 +7273,10 @@
         <v>32</v>
       </c>
       <c r="C157" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D157" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E157" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -7254,7 +7291,7 @@
         <v>1.26</v>
       </c>
       <c r="H157" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I157" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7273,10 +7310,10 @@
         <v>32</v>
       </c>
       <c r="C158" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D158" s="6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E158" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -7291,7 +7328,7 @@
         <v>1.26</v>
       </c>
       <c r="H158" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I158" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7307,7 +7344,7 @@
       <c r="B159" s="31"/>
       <c r="C159" s="31"/>
       <c r="D159" s="11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E159" s="31"/>
       <c r="F159" s="31"/>
@@ -7341,10 +7378,10 @@
         <v>33</v>
       </c>
       <c r="C162" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D162" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E162" s="26" t="n">
         <v>0.15</v>
@@ -7358,7 +7395,7 @@
         <v>0.15</v>
       </c>
       <c r="H162" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I162" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7377,10 +7414,10 @@
         <v>33</v>
       </c>
       <c r="C163" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D163" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E163" s="26" t="n">
         <v>1.75</v>
@@ -7394,7 +7431,7 @@
         <v>1.75</v>
       </c>
       <c r="H163" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I163" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7413,10 +7450,10 @@
         <v>33</v>
       </c>
       <c r="C164" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D164" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E164" s="26" t="n">
         <v>0.15</v>
@@ -7430,7 +7467,7 @@
         <v>0.15</v>
       </c>
       <c r="H164" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I164" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7449,10 +7486,10 @@
         <v>33</v>
       </c>
       <c r="C165" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D165" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E165" s="26" t="n">
         <v>1.75</v>
@@ -7466,7 +7503,7 @@
         <v>1.75</v>
       </c>
       <c r="H165" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I165" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7485,10 +7522,10 @@
         <v>33</v>
       </c>
       <c r="C166" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D166" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E166" s="26" t="n">
         <v>6.3</v>
@@ -7502,7 +7539,7 @@
         <v>22.05</v>
       </c>
       <c r="H166" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I166" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7521,10 +7558,10 @@
         <v>33</v>
       </c>
       <c r="C167" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D167" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E167" s="26" t="n">
         <v>0.15</v>
@@ -7538,7 +7575,7 @@
         <v>0.525</v>
       </c>
       <c r="H167" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I167" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7557,10 +7594,10 @@
         <v>33</v>
       </c>
       <c r="C168" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D168" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E168" s="26" t="n">
         <v>1.5</v>
@@ -7574,7 +7611,7 @@
         <v>1.5</v>
       </c>
       <c r="H168" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I168" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7593,10 +7630,10 @@
         <v>33</v>
       </c>
       <c r="C169" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D169" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E169" s="26" t="n">
         <v>0.2</v>
@@ -7610,7 +7647,7 @@
         <v>0.7</v>
       </c>
       <c r="H169" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I169" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7629,10 +7666,10 @@
         <v>33</v>
       </c>
       <c r="C170" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D170" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E170" s="26" t="n">
         <v>4.7</v>
@@ -7646,7 +7683,7 @@
         <v>4.7</v>
       </c>
       <c r="H170" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I170" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7665,10 +7702,10 @@
         <v>33</v>
       </c>
       <c r="C171" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D171" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E171" s="26" t="n">
         <v>0.4</v>
@@ -7682,7 +7719,7 @@
         <v>1.4</v>
       </c>
       <c r="H171" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I171" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7701,10 +7738,10 @@
         <v>33</v>
       </c>
       <c r="C172" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D172" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E172" s="26" t="n">
         <v>4.7</v>
@@ -7718,7 +7755,7 @@
         <v>4.7</v>
       </c>
       <c r="H172" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I172" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7737,10 +7774,10 @@
         <v>33</v>
       </c>
       <c r="C173" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D173" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E173" s="26" t="n">
         <v>0.35</v>
@@ -7754,7 +7791,7 @@
         <v>1.225</v>
       </c>
       <c r="H173" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I173" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7773,10 +7810,10 @@
         <v>33</v>
       </c>
       <c r="C174" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D174" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E174" s="26" t="n">
         <v>0.1</v>
@@ -7790,7 +7827,7 @@
         <v>0.35</v>
       </c>
       <c r="H174" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I174" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7809,10 +7846,10 @@
         <v>33</v>
       </c>
       <c r="C175" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D175" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E175" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -7827,7 +7864,7 @@
         <v>1.26</v>
       </c>
       <c r="H175" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I175" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7846,10 +7883,10 @@
         <v>33</v>
       </c>
       <c r="C176" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D176" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E176" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -7864,7 +7901,7 @@
         <v>1.26</v>
       </c>
       <c r="H176" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I176" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7883,10 +7920,10 @@
         <v>33</v>
       </c>
       <c r="C177" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D177" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E177" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -7901,7 +7938,7 @@
         <v>1.26</v>
       </c>
       <c r="H177" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I177" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7920,10 +7957,10 @@
         <v>33</v>
       </c>
       <c r="C178" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D178" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E178" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -7938,7 +7975,7 @@
         <v>1.26</v>
       </c>
       <c r="H178" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I178" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7957,10 +7994,10 @@
         <v>33</v>
       </c>
       <c r="C179" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D179" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E179" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -7975,7 +8012,7 @@
         <v>1.26</v>
       </c>
       <c r="H179" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I179" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -7994,10 +8031,10 @@
         <v>33</v>
       </c>
       <c r="C180" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D180" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E180" s="7" t="n">
         <f aca="false">Narxlar!$C$16</f>
@@ -8012,7 +8049,7 @@
         <v>1.26</v>
       </c>
       <c r="H180" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I180" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -8028,7 +8065,7 @@
       <c r="B181" s="31"/>
       <c r="C181" s="31"/>
       <c r="D181" s="11" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E181" s="31"/>
       <c r="F181" s="31"/>
@@ -8062,10 +8099,10 @@
         <v>34</v>
       </c>
       <c r="C184" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D184" s="6" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E184" s="26" t="n">
         <v>0.4</v>
@@ -8079,7 +8116,7 @@
         <v>1.4</v>
       </c>
       <c r="H184" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I184" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -8098,10 +8135,10 @@
         <v>34</v>
       </c>
       <c r="C185" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D185" s="6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E185" s="26" t="n">
         <v>0.7</v>
@@ -8115,7 +8152,7 @@
         <v>2.45</v>
       </c>
       <c r="H185" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I185" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -8134,10 +8171,10 @@
         <v>34</v>
       </c>
       <c r="C186" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D186" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E186" s="26" t="n">
         <v>1.65</v>
@@ -8151,7 +8188,7 @@
         <v>5.775</v>
       </c>
       <c r="H186" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I186" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -8167,7 +8204,7 @@
       <c r="B187" s="31"/>
       <c r="C187" s="31"/>
       <c r="D187" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E187" s="31"/>
       <c r="F187" s="31"/>
@@ -8201,10 +8238,10 @@
         <v>35</v>
       </c>
       <c r="C190" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D190" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E190" s="26" t="n">
         <v>2.6</v>
@@ -8218,7 +8255,7 @@
         <v>9.1</v>
       </c>
       <c r="H190" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I190" s="28" t="n">
         <f aca="false">Narxlar!$C$6</f>
@@ -8234,7 +8271,7 @@
       <c r="B191" s="31"/>
       <c r="C191" s="31"/>
       <c r="D191" s="11" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E191" s="31"/>
       <c r="F191" s="31"/>
@@ -8271,7 +8308,7 @@
         <v>56</v>
       </c>
       <c r="D194" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E194" s="7" t="n">
         <f aca="false">Narxlar!$C$10</f>
@@ -8299,7 +8336,7 @@
       <c r="B195" s="31"/>
       <c r="C195" s="31"/>
       <c r="D195" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E195" s="31"/>
       <c r="F195" s="31"/>
@@ -8333,60 +8370,205 @@
         <v>22</v>
       </c>
       <c r="C198" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D198" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="E198" s="26" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="F198" s="7" t="n">
+        <f aca="false">Narxlar!$C$18</f>
+        <v>2.5</v>
+      </c>
+      <c r="G198" s="27" t="n">
+        <f aca="false">E198*F198</f>
+        <v>13.625</v>
+      </c>
+      <c r="H198" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="I198" s="28" t="n">
+        <f aca="false">Narxlar!$C$7</f>
+        <v>15.5</v>
+      </c>
+      <c r="J198" s="29" t="n">
+        <f aca="false">G198*I198</f>
+        <v>211.1875</v>
+      </c>
+    </row>
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="20" t="n">
+        <v>143</v>
+      </c>
+      <c r="B199" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C199" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D199" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="E199" s="26" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="F199" s="7" t="n">
+        <f aca="false">Narxlar!$C$18</f>
+        <v>2.5</v>
+      </c>
+      <c r="G199" s="27" t="n">
+        <f aca="false">E199*F199</f>
+        <v>13.625</v>
+      </c>
+      <c r="H199" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="I199" s="28" t="n">
+        <f aca="false">Narxlar!$C$7</f>
+        <v>15.5</v>
+      </c>
+      <c r="J199" s="29" t="n">
+        <f aca="false">G199*I199</f>
+        <v>211.1875</v>
+      </c>
+    </row>
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="20" t="n">
+        <v>144</v>
+      </c>
+      <c r="B200" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C200" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D200" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="E200" s="26" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="F200" s="7" t="n">
+        <f aca="false">Narxlar!$C$18</f>
+        <v>2.5</v>
+      </c>
+      <c r="G200" s="27" t="n">
+        <f aca="false">E200*F200</f>
+        <v>21.5</v>
+      </c>
+      <c r="H200" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="I200" s="28" t="n">
+        <f aca="false">Narxlar!$C$7</f>
+        <v>15.5</v>
+      </c>
+      <c r="J200" s="29" t="n">
+        <f aca="false">G200*I200</f>
+        <v>333.25</v>
+      </c>
+    </row>
+    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="20" t="n">
+        <v>145</v>
+      </c>
+      <c r="B201" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C201" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D201" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="E201" s="7" t="n">
+        <f aca="false">Narxlar!$C$16</f>
+        <v>0.9</v>
+      </c>
+      <c r="F201" s="7" t="n">
+        <f aca="false">Narxlar!$C$14</f>
+        <v>2.1</v>
+      </c>
+      <c r="G201" s="27" t="n">
+        <f aca="false">-E201*F201</f>
+        <v>-1.89</v>
+      </c>
+      <c r="H201" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="I201" s="28" t="n">
+        <f aca="false">Narxlar!$C$7</f>
+        <v>15.5</v>
+      </c>
+      <c r="J201" s="29" t="n">
+        <f aca="false">G201*I201</f>
+        <v>-29.295</v>
+      </c>
+    </row>
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="20" t="n">
+        <v>146</v>
+      </c>
+      <c r="B202" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C202" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D198" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="E198" s="26"/>
-      <c r="F198" s="27"/>
-      <c r="G198" s="30" t="n">
+      <c r="D202" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="E202" s="26"/>
+      <c r="F202" s="27"/>
+      <c r="G202" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="H198" s="20" t="s">
-        <v>102</v>
-      </c>
-      <c r="I198" s="28" t="n">
+      <c r="H202" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="I202" s="28" t="n">
         <f aca="false">Narxlar!$C$8</f>
         <v>1032</v>
       </c>
-      <c r="J198" s="29" t="n">
-        <f aca="false">G198*I198</f>
+      <c r="J202" s="29" t="n">
+        <f aca="false">G202*I202</f>
         <v>1032</v>
       </c>
     </row>
-    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A199" s="31"/>
-      <c r="B199" s="31"/>
-      <c r="C199" s="31"/>
-      <c r="D199" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="E199" s="31"/>
-      <c r="F199" s="31"/>
-      <c r="G199" s="31"/>
-      <c r="H199" s="31"/>
-      <c r="I199" s="31"/>
-      <c r="J199" s="32" t="n">
-        <f aca="false">SUM(J198:J198)</f>
-        <v>1032</v>
-      </c>
-    </row>
-    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A201" s="31"/>
-      <c r="B201" s="31"/>
-      <c r="C201" s="31"/>
-      <c r="D201" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="E201" s="31"/>
-      <c r="F201" s="31"/>
-      <c r="G201" s="31"/>
-      <c r="H201" s="31"/>
-      <c r="I201" s="31"/>
-      <c r="J201" s="32" t="n">
-        <f aca="false">J14+J24+J33+J52+J62+J74+J87+J100+J113+J124+J135+J141+J159+J181+J187+J191+J195+J199</f>
-        <v>27845.245</v>
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="31"/>
+      <c r="B203" s="31"/>
+      <c r="C203" s="31"/>
+      <c r="D203" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="E203" s="31"/>
+      <c r="F203" s="31"/>
+      <c r="G203" s="31"/>
+      <c r="H203" s="31"/>
+      <c r="I203" s="31"/>
+      <c r="J203" s="32" t="n">
+        <f aca="false">SUM(J198:J202)</f>
+        <v>1758.33</v>
+      </c>
+    </row>
+    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="31"/>
+      <c r="B205" s="31"/>
+      <c r="C205" s="31"/>
+      <c r="D205" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="E205" s="31"/>
+      <c r="F205" s="31"/>
+      <c r="G205" s="31"/>
+      <c r="H205" s="31"/>
+      <c r="I205" s="31"/>
+      <c r="J205" s="32" t="n">
+        <f aca="false">J14+J24+J33+J52+J62+J74+J87+J100+J113+J124+J135+J141+J159+J181+J187+J191+J195+J203</f>
+        <v>28571.575</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Xadra xarajatlar: dollar kursi 11 900 so'm
Buyurtmachi kursi bo'yicha so'mdagi ishlar qayta hisoblandi.
Umumiy jami 44 308.91 $ (≈ 527.3 mln so'm).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0121VSEFiRNp3h6KMycRzKQh
</commit_message>
<xml_diff>
--- a/xadra-filiali/hisob/Xadra_2-qavat_xarajatlar_v1.0.xlsx
+++ b/xadra-filiali/hisob/Xadra_2-qavat_xarajatlar_v1.0.xlsx
@@ -282,7 +282,7 @@
     <t xml:space="preserve">so'm/$</t>
   </si>
   <si>
-    <t xml:space="preserve">TAXMIN — joriy kursni yozing; so'mdagi narxlar shu kurs bo'yicha $ ga o'tadi</t>
+    <t xml:space="preserve">Buyurtmachi; so'mdagi narxlar shu kurs bo'yicha $ ga o'tadi</t>
   </si>
   <si>
     <t xml:space="preserve">Matli plyonka (shisha devorga)</t>
@@ -393,7 +393,7 @@
     <t xml:space="preserve">• Videokuzatuv: 16 ta kamera (40 $) va o'rnatish (21 $ dan), NVR, kabellar jami; logotiplar jami — «Butun qavat» qatorida.</t>
   </si>
   <si>
-    <t xml:space="preserve">• So'mdagi narxlar (matli plyonka, yong'in xavfsizligi, devor buzish va chiqindi) «Dollar kursi» katagi bo'yicha $ ga o'tkaziladi — kursni tekshiring.</t>
+    <t xml:space="preserve">• So'mdagi narxlar (matli plyonka, yong'in xavfsizligi, devor buzish va chiqindi) «Dollar kursi» katagi bo'yicha (11 900 so'm/$) $ ga o'tkaziladi.</t>
   </si>
   <si>
     <t xml:space="preserve">• Devor buzish: chizmadagi buziladigan devorlar uzunligi × devor balandligi (3.5 m) × 50 000 so'm/m².</t>
@@ -3031,19 +3031,19 @@
       </c>
       <c r="O30" s="8" t="n">
         <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$257,'Hisob (batafsil)'!$B$5:$B$257,$A30,'Hisob (batafsil)'!$C$5:$C$257,"Matli plyonka")</f>
-        <v>503.937007874016</v>
+        <v>537.81512605042</v>
       </c>
       <c r="P30" s="8" t="n">
         <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$257,'Hisob (batafsil)'!$B$5:$B$257,$A30,'Hisob (batafsil)'!$C$5:$C$257,"Yong'in xavfsizligi")</f>
-        <v>1417.32283464567</v>
+        <v>1512.60504201681</v>
       </c>
       <c r="Q30" s="8" t="n">
         <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$257,'Hisob (batafsil)'!$B$5:$B$257,$A30,'Hisob (batafsil)'!$C$5:$C$257,"Buzish ishlari")</f>
-        <v>423.129921259843</v>
+        <v>451.575630252101</v>
       </c>
       <c r="R30" s="10" t="n">
         <f aca="false">C30+E30+G30+I30+K30+L30+M30+N30+O30+P30+Q30</f>
-        <v>6963.38976377953</v>
+        <v>7120.99579831933</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3104,19 +3104,19 @@
       </c>
       <c r="O31" s="13" t="n">
         <f aca="false">SUM(O25:O30)</f>
-        <v>503.937007874016</v>
+        <v>537.81512605042</v>
       </c>
       <c r="P31" s="13" t="n">
         <f aca="false">SUM(P25:P30)</f>
-        <v>1417.32283464567</v>
+        <v>1512.60504201681</v>
       </c>
       <c r="Q31" s="13" t="n">
         <f aca="false">SUM(Q25:Q30)</f>
-        <v>423.129921259843</v>
+        <v>451.575630252101</v>
       </c>
       <c r="R31" s="13" t="n">
         <f aca="false">SUM(R25:R30)</f>
-        <v>11312.7897637795</v>
+        <v>11470.3957983193</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3177,19 +3177,19 @@
       </c>
       <c r="O33" s="17" t="n">
         <f aca="false">O14+O22+O31</f>
-        <v>503.937007874016</v>
+        <v>537.81512605042</v>
       </c>
       <c r="P33" s="17" t="n">
         <f aca="false">P14+P22+P31</f>
-        <v>1417.32283464567</v>
+        <v>1512.60504201681</v>
       </c>
       <c r="Q33" s="17" t="n">
         <f aca="false">Q14+Q22+Q31</f>
-        <v>423.129921259843</v>
+        <v>451.575630252101</v>
       </c>
       <c r="R33" s="17" t="n">
         <f aca="false">R14+R22+R31</f>
-        <v>40123.2247637795</v>
+        <v>40280.8307983193</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3215,7 +3215,7 @@
       <c r="Q34" s="19"/>
       <c r="R34" s="20" t="n">
         <f aca="false">R33*Narxlar!$C$25</f>
-        <v>4012.32247637795</v>
+        <v>4028.08307983193</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3240,7 +3240,7 @@
       <c r="Q35" s="15"/>
       <c r="R35" s="17" t="n">
         <f aca="false">R33+R34</f>
-        <v>44135.5472401575</v>
+        <v>44308.9138781513</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3265,7 +3265,7 @@
       <c r="Q36" s="15"/>
       <c r="R36" s="21" t="n">
         <f aca="false">R35*Narxlar!$C$19</f>
-        <v>560521449.95</v>
+        <v>527276075.15</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3581,7 +3581,7 @@
         <v>84</v>
       </c>
       <c r="C19" s="27" t="n">
-        <v>12700</v>
+        <v>11900</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>85</v>
@@ -10864,11 +10864,11 @@
       </c>
       <c r="I236" s="34" t="n">
         <f aca="false">Narxlar!$C$20/Narxlar!$C$19</f>
-        <v>62.992125984252</v>
+        <v>67.2268907563025</v>
       </c>
       <c r="J236" s="35" t="n">
         <f aca="false">G236*I236</f>
-        <v>503.937007874016</v>
+        <v>537.81512605042</v>
       </c>
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10894,11 +10894,11 @@
       </c>
       <c r="I237" s="34" t="n">
         <f aca="false">Narxlar!$C$22/Narxlar!$C$19</f>
-        <v>1417.32283464567</v>
+        <v>1512.60504201681</v>
       </c>
       <c r="J237" s="35" t="n">
         <f aca="false">G237*I237</f>
-        <v>1417.32283464567</v>
+        <v>1512.60504201681</v>
       </c>
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10930,11 +10930,11 @@
       </c>
       <c r="I238" s="34" t="n">
         <f aca="false">Narxlar!$C$23/Narxlar!$C$19</f>
-        <v>3.93700787401575</v>
+        <v>4.20168067226891</v>
       </c>
       <c r="J238" s="35" t="n">
         <f aca="false">G238*I238</f>
-        <v>15.1574803149606</v>
+        <v>16.1764705882353</v>
       </c>
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10966,11 +10966,11 @@
       </c>
       <c r="I239" s="34" t="n">
         <f aca="false">Narxlar!$C$23/Narxlar!$C$19</f>
-        <v>3.93700787401575</v>
+        <v>4.20168067226891</v>
       </c>
       <c r="J239" s="35" t="n">
         <f aca="false">G239*I239</f>
-        <v>77.1653543307087</v>
+        <v>82.3529411764706</v>
       </c>
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11002,11 +11002,11 @@
       </c>
       <c r="I240" s="34" t="n">
         <f aca="false">Narxlar!$C$23/Narxlar!$C$19</f>
-        <v>3.93700787401575</v>
+        <v>4.20168067226891</v>
       </c>
       <c r="J240" s="35" t="n">
         <f aca="false">G240*I240</f>
-        <v>77.1653543307087</v>
+        <v>82.3529411764706</v>
       </c>
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11038,11 +11038,11 @@
       </c>
       <c r="I241" s="34" t="n">
         <f aca="false">Narxlar!$C$23/Narxlar!$C$19</f>
-        <v>3.93700787401575</v>
+        <v>4.20168067226891</v>
       </c>
       <c r="J241" s="35" t="n">
         <f aca="false">G241*I241</f>
-        <v>10.3346456692913</v>
+        <v>11.0294117647059</v>
       </c>
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11074,11 +11074,11 @@
       </c>
       <c r="I242" s="34" t="n">
         <f aca="false">Narxlar!$C$23/Narxlar!$C$19</f>
-        <v>3.93700787401575</v>
+        <v>4.20168067226891</v>
       </c>
       <c r="J242" s="35" t="n">
         <f aca="false">G242*I242</f>
-        <v>46.8503937007874</v>
+        <v>50</v>
       </c>
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11110,11 +11110,11 @@
       </c>
       <c r="I243" s="34" t="n">
         <f aca="false">Narxlar!$C$23/Narxlar!$C$19</f>
-        <v>3.93700787401575</v>
+        <v>4.20168067226891</v>
       </c>
       <c r="J243" s="35" t="n">
         <f aca="false">G243*I243</f>
-        <v>57.8740157480315</v>
+        <v>61.764705882353</v>
       </c>
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11146,11 +11146,11 @@
       </c>
       <c r="I244" s="34" t="n">
         <f aca="false">Narxlar!$C$23/Narxlar!$C$19</f>
-        <v>3.93700787401575</v>
+        <v>4.20168067226891</v>
       </c>
       <c r="J244" s="35" t="n">
         <f aca="false">G244*I244</f>
-        <v>20.6692913385827</v>
+        <v>22.0588235294118</v>
       </c>
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11182,11 +11182,11 @@
       </c>
       <c r="I245" s="34" t="n">
         <f aca="false">Narxlar!$C$23/Narxlar!$C$19</f>
-        <v>3.93700787401575</v>
+        <v>4.20168067226891</v>
       </c>
       <c r="J245" s="35" t="n">
         <f aca="false">G245*I245</f>
-        <v>2.75590551181102</v>
+        <v>2.94117647058824</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11218,11 +11218,11 @@
       </c>
       <c r="I246" s="34" t="n">
         <f aca="false">Narxlar!$C$23/Narxlar!$C$19</f>
-        <v>3.93700787401575</v>
+        <v>4.20168067226891</v>
       </c>
       <c r="J246" s="35" t="n">
         <f aca="false">G246*I246</f>
-        <v>20.6692913385827</v>
+        <v>22.0588235294118</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11248,11 +11248,11 @@
       </c>
       <c r="I247" s="34" t="n">
         <f aca="false">Narxlar!$C$24/Narxlar!$C$19</f>
-        <v>94.488188976378</v>
+        <v>100.840336134454</v>
       </c>
       <c r="J247" s="35" t="n">
         <f aca="false">G247*I247</f>
-        <v>94.488188976378</v>
+        <v>100.840336134454</v>
       </c>
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11269,7 +11269,7 @@
       <c r="I248" s="37"/>
       <c r="J248" s="38" t="n">
         <f aca="false">SUM(J231:J247)</f>
-        <v>6963.38976377953</v>
+        <v>7120.99579831933</v>
       </c>
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11492,7 +11492,7 @@
       <c r="I258" s="37"/>
       <c r="J258" s="38" t="n">
         <f aca="false">J16+J28+J39+J60+J72+J86+J101+J116+J131+J146+J161+J168+J190+J213+J220+J224+J228+J248+J256</f>
-        <v>40123.2247637795</v>
+        <v>40280.8307983193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>